<commit_message>
Update Excel with all 41 objects and 6 permission sets from repo
Single-cell comma-separated format: Read,Create,Edit,Delete,View All,Modify All
Includes standard objects, custom objects, metadata types, and custom settings.

https://claude.ai/code/session_01W7w6NEfmrmVUma43ot3fAT
</commit_message>
<xml_diff>
--- a/Object_Permissions_By_PermissionSet.xlsx
+++ b/Object_Permissions_By_PermissionSet.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Object Permissions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tab Access" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -79,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -88,11 +89,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -462,12 +466,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -503,7 +507,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>sfdc_scrt2</t>
+          <t>sfdc_scrt2 (SCRT2 Integration)</t>
         </is>
       </c>
     </row>
@@ -523,50 +527,66 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Apex_Log__c</t>
+          <t>Contact</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr"/>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
-      <c r="F3" s="3" t="inlineStr"/>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
       <c r="G3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Architect__c</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr"/>
-      <c r="C4" s="3" t="inlineStr"/>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Read,Create,Edit,Delete,View All,Modify All</t>
-        </is>
-      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Read,Create,Edit</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr"/>
-      <c r="F4" s="3" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
       <c r="G4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Campaign</t>
+          <t>Opportunity</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr"/>
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
       <c r="F5" s="3" t="inlineStr"/>
       <c r="G5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Cart__c</t>
+          <t>OpportunityLineItem</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr"/>
@@ -579,7 +599,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Cart_Line_Item__c</t>
+          <t>Order</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr"/>
@@ -592,7 +612,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Case</t>
+          <t>OrderItem</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr"/>
@@ -600,16 +620,12 @@
       <c r="D8" s="3" t="inlineStr"/>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="3" t="inlineStr"/>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>Read,View All</t>
-        </is>
-      </c>
+      <c r="G8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Collection_Visit__c</t>
+          <t>Product2</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr"/>
@@ -622,7 +638,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Contact</t>
+          <t>Quote</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr"/>
@@ -630,20 +646,16 @@
       <c r="D10" s="3" t="inlineStr"/>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Read</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>Read</t>
-        </is>
-      </c>
+          <t>Read,Create,Edit</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr"/>
       <c r="G10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Customer__c</t>
+          <t>QuoteLineItem</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr"/>
@@ -656,7 +668,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Deals__c</t>
+          <t>Case</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr"/>
@@ -664,12 +676,16 @@
       <c r="D12" s="3" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="3" t="inlineStr"/>
-      <c r="G12" s="3" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Read,View All</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Delivery_Group__c</t>
+          <t>Campaign</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr"/>
@@ -682,7 +698,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Delivery_Line_Item__c</t>
+          <t>Apex_Log__c</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr"/>
@@ -695,12 +711,16 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Engagement__c</t>
+          <t>Architect__c</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr"/>
       <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr"/>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Read,Create,Edit,Delete,View All,Modify All</t>
+        </is>
+      </c>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="3" t="inlineStr"/>
       <c r="G15" s="3" t="inlineStr"/>
@@ -708,7 +728,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Finance_Transactions__c</t>
+          <t>Cart__c</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr"/>
@@ -721,7 +741,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Firm__c</t>
+          <t>Cart_Line_Item__c</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr"/>
@@ -734,7 +754,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>In_App_Checklist_Settings__c</t>
+          <t>Collection_Visit__c</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr"/>
@@ -747,7 +767,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Integration_Config__mdt</t>
+          <t>Customer__c</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr"/>
@@ -760,7 +780,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Invoice__c</t>
+          <t>Deals__c</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr"/>
@@ -773,7 +793,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Invoice_Item__c</t>
+          <t>Delivery_Group__c</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr"/>
@@ -786,45 +806,33 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Delivery_Line_Item__c</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr"/>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Read,Create,Edit</t>
-        </is>
-      </c>
+      <c r="C22" s="3" t="inlineStr"/>
       <c r="D22" s="3" t="inlineStr"/>
       <c r="E22" s="3" t="inlineStr"/>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>Read</t>
-        </is>
-      </c>
+      <c r="F22" s="3" t="inlineStr"/>
       <c r="G22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Opportunity</t>
+          <t>Engagement__c</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr"/>
       <c r="C23" s="3" t="inlineStr"/>
       <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>Read</t>
-        </is>
-      </c>
+      <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="3" t="inlineStr"/>
       <c r="G23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>OpportunityLineItem</t>
+          <t>Finance_Transactions__c</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr"/>
@@ -837,7 +845,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Order</t>
+          <t>Firm__c</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr"/>
@@ -850,7 +858,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>OrderItem</t>
+          <t>Invoice__c</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr"/>
@@ -863,7 +871,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Order_Batch_Item__c</t>
+          <t>Invoice_Item__c</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr"/>
@@ -876,7 +884,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Payment__c</t>
+          <t>Order_Batch_Item__c</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr"/>
@@ -889,7 +897,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Pending_Purchase__c</t>
+          <t>Payment__c</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr"/>
@@ -902,7 +910,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Pending_Purchase_Line_Item__c</t>
+          <t>Pending_Purchase__c</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr"/>
@@ -915,7 +923,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Product2</t>
+          <t>Pending_Purchase_Line_Item__c</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr"/>
@@ -941,7 +949,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Product_Sync_Setting__c</t>
+          <t>Projects__c</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr"/>
@@ -954,7 +962,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Projects__c</t>
+          <t>Sales_Confirmation__c</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr"/>
@@ -967,29 +975,29 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Quote</t>
+          <t>Vendor__c</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr"/>
       <c r="C35" s="3" t="inlineStr"/>
       <c r="D35" s="3" t="inlineStr"/>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>Read,Create,Edit</t>
-        </is>
-      </c>
+      <c r="E35" s="3" t="inlineStr"/>
       <c r="F35" s="3" t="inlineStr"/>
       <c r="G35" s="3" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>QuoteLineItem</t>
+          <t>Warehouse__c</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr"/>
       <c r="C36" s="3" t="inlineStr"/>
-      <c r="D36" s="3" t="inlineStr"/>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Read,Create,Edit,Delete,View All,Modify All</t>
+        </is>
+      </c>
       <c r="E36" s="3" t="inlineStr"/>
       <c r="F36" s="3" t="inlineStr"/>
       <c r="G36" s="3" t="inlineStr"/>
@@ -997,12 +1005,16 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Sales_Confirmation__c</t>
+          <t>Wishlist_Item__c</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr"/>
       <c r="C37" s="3" t="inlineStr"/>
-      <c r="D37" s="3" t="inlineStr"/>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Read,Create,Edit,Delete,View All,Modify All</t>
+        </is>
+      </c>
       <c r="E37" s="3" t="inlineStr"/>
       <c r="F37" s="3" t="inlineStr"/>
       <c r="G37" s="3" t="inlineStr"/>
@@ -1010,7 +1022,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>SAP_Config__mdt</t>
+          <t>Integration_Config__mdt</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr"/>
@@ -1023,7 +1035,7 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>SAP_Sync_Setting__c</t>
+          <t>SAP_Config__mdt</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr"/>
@@ -1036,7 +1048,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Vendor__c</t>
+          <t>In_App_Checklist_Settings__c</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr"/>
@@ -1049,16 +1061,12 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Warehouse__c</t>
+          <t>Product_Sync_Setting__c</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr"/>
       <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>Read,Create,Edit,Delete,View All,Modify All</t>
-        </is>
-      </c>
+      <c r="D41" s="3" t="inlineStr"/>
       <c r="E41" s="3" t="inlineStr"/>
       <c r="F41" s="3" t="inlineStr"/>
       <c r="G41" s="3" t="inlineStr"/>
@@ -1066,19 +1074,109 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Wishlist_Item__c</t>
+          <t>SAP_Sync_Setting__c</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr"/>
       <c r="C42" s="3" t="inlineStr"/>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>Read,Create,Edit,Delete,View All,Modify All</t>
-        </is>
-      </c>
+      <c r="D42" s="3" t="inlineStr"/>
       <c r="E42" s="3" t="inlineStr"/>
       <c r="F42" s="3" t="inlineStr"/>
       <c r="G42" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Tab Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Sales_User</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Salesforce_Lead_Capture</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Field_Visible</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Quotation_Email_Access</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>sfdc_activityplatform</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>sfdc_scrt2 (SCRT2 Integration)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Architect__c</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr"/>
+      <c r="C2" s="6" t="inlineStr"/>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>Visible</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr"/>
+      <c r="F2" s="6" t="inlineStr"/>
+      <c r="G2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Wishlist_Item__c</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr"/>
+      <c r="C3" s="6" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Visible</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr"/>
+      <c r="F3" s="6" t="inlineStr"/>
+      <c r="G3" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>